<commit_message>
Add CozyYard Luban table generators for tree, order, expansion, and shop.
Include ##type schema rows and read_schema_from_file so Luban can load bean definitions from Excel.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Luban/DataTables/Datas/CozyYard/__tables__.xlsx
+++ b/Tools/Luban/DataTables/Datas/CozyYard/__tables__.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">

</xml_diff>

<commit_message>
Add Luban TbWeather config table for season weather probabilities.
Includes weather.xlsx generator, table registration, and regenerated Tables/TablesExt.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Luban/DataTables/Datas/CozyYard/__tables__.xlsx
+++ b/Tools/Luban/DataTables/Datas/CozyYard/__tables__.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1159,6 +1159,47 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TbWeather</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>weather.xlsx</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>天气配置表</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>